<commit_message>
show excel on site
</commit_message>
<xml_diff>
--- a/stock_details.xlsx
+++ b/stock_details.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -508,10 +508,10 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>25</v>
+        <v>25.1</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>759</v>
@@ -523,10 +523,10 @@
         <v>13.4</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-33.72859025032938</v>
+        <v>-33.59683794466403</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>12.78026905829596</v>
+        <v>13.00448430493273</v>
       </c>
     </row>
     <row r="3">
@@ -536,10 +536,10 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>26.6</v>
+        <v>26.1</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1259</v>
+        <v>1234</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>1621</v>
@@ -551,10 +551,10 @@
         <v>12.9</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-22.33189389265885</v>
+        <v>-23.87415175817397</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>27.55825734549139</v>
+        <v>25.02532928064843</v>
       </c>
     </row>
     <row r="4">
@@ -567,7 +567,7 @@
         <v>10.2</v>
       </c>
       <c r="C4" t="n">
-        <v>1362</v>
+        <v>1350</v>
       </c>
       <c r="D4" t="n">
         <v>2680</v>
@@ -579,10 +579,10 @@
         <v>21.9</v>
       </c>
       <c r="G4" t="n">
-        <v>-49.17910447761194</v>
+        <v>-49.62686567164179</v>
       </c>
       <c r="H4" t="n">
-        <v>16.01362862010222</v>
+        <v>14.99148211243612</v>
       </c>
     </row>
     <row r="5">
@@ -592,10 +592,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>13.1</v>
+        <v>12.7</v>
       </c>
       <c r="C5" t="n">
-        <v>1185</v>
+        <v>1147</v>
       </c>
       <c r="D5" t="n">
         <v>1340</v>
@@ -607,10 +607,10 @@
         <v>7.06</v>
       </c>
       <c r="G5" t="n">
-        <v>-11.56716417910448</v>
+        <v>-14.40298507462686</v>
       </c>
       <c r="H5" t="n">
-        <v>18.97590361445783</v>
+        <v>15.16064257028112</v>
       </c>
     </row>
     <row r="6">
@@ -620,25 +620,25 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>34.5</v>
+        <v>34.4</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>9100</v>
+        <v>9070</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>12774</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>6018</v>
+        <v>6224</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>33.5</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>-28.76154689212463</v>
+        <v>-28.9963989353374</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>51.21302758391493</v>
+        <v>45.72622107969151</v>
       </c>
     </row>
     <row r="7">
@@ -648,10 +648,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10.2</v>
+        <v>10.1</v>
       </c>
       <c r="C7" t="n">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D7" t="n">
         <v>263</v>
@@ -663,10 +663,10 @@
         <v>7.06</v>
       </c>
       <c r="G7" t="n">
-        <v>-33.07984790874524</v>
+        <v>-33.84030418250951</v>
       </c>
       <c r="H7" t="n">
-        <v>7.975460122699387</v>
+        <v>6.748466257668712</v>
       </c>
     </row>
     <row r="8">
@@ -676,10 +676,10 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="D8" s="4" t="n">
         <v>335</v>
@@ -691,10 +691,10 @@
         <v>3.37</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-25.67164179104477</v>
+        <v>-24.17910447761194</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>50</v>
+        <v>53.01204819277109</v>
       </c>
     </row>
     <row r="9">
@@ -704,13 +704,13 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>73.90000000000001</v>
+        <v>75.7</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>1884</v>
+        <v>1930</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>1899</v>
+        <v>1935</v>
       </c>
       <c r="E9" s="4" t="n">
         <v>811</v>
@@ -719,10 +719,10 @@
         <v>40.2</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>-0.7898894154818324</v>
+        <v>-0.2583979328165375</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>132.3057953144266</v>
+        <v>137.9778051787916</v>
       </c>
     </row>
     <row r="10">
@@ -732,10 +732,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>15.2</v>
+        <v>15</v>
       </c>
       <c r="C10" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D10" t="n">
         <v>76.90000000000001</v>
@@ -747,10 +747,10 @@
         <v>5.29</v>
       </c>
       <c r="G10" t="n">
-        <v>-21.97659297789338</v>
+        <v>-23.27698309492848</v>
       </c>
       <c r="H10" t="n">
-        <v>29.87012987012986</v>
+        <v>27.7056277056277</v>
       </c>
     </row>
     <row r="11">
@@ -760,10 +760,10 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>25.9</v>
+        <v>25.5</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>1477</v>
+        <v>1454</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>1702</v>
@@ -775,10 +775,10 @@
         <v>22.8</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>-13.21974148061105</v>
+        <v>-14.5710928319624</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>23.90939597315436</v>
+        <v>21.97986577181208</v>
       </c>
     </row>
     <row r="12">
@@ -791,10 +791,10 @@
         <v>13</v>
       </c>
       <c r="C12" t="n">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D12" t="n">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E12" t="n">
         <v>125</v>
@@ -803,10 +803,10 @@
         <v>6.57</v>
       </c>
       <c r="G12" t="n">
-        <v>-1.06951871657754</v>
+        <v>-1.063829787234043</v>
       </c>
       <c r="H12" t="n">
-        <v>48</v>
+        <v>48.8</v>
       </c>
     </row>
     <row r="13">
@@ -816,10 +816,10 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>31.7</v>
+        <v>31.3</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>426</v>
+        <v>420</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>582</v>
@@ -831,10 +831,10 @@
         <v>46</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>-26.80412371134021</v>
+        <v>-27.83505154639175</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>4.926108374384237</v>
+        <v>3.448275862068965</v>
       </c>
     </row>
     <row r="14">
@@ -844,25 +844,25 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>19.6</v>
+        <v>19.4</v>
       </c>
       <c r="C14" t="n">
-        <v>1254</v>
+        <v>1239</v>
       </c>
       <c r="D14" t="n">
         <v>1421</v>
       </c>
       <c r="E14" t="n">
-        <v>1074</v>
+        <v>1094</v>
       </c>
       <c r="F14" t="n">
         <v>26.5</v>
       </c>
       <c r="G14" t="n">
-        <v>-11.75228712174525</v>
+        <v>-12.80788177339902</v>
       </c>
       <c r="H14" t="n">
-        <v>16.75977653631285</v>
+        <v>13.25411334552102</v>
       </c>
     </row>
     <row r="15">
@@ -872,10 +872,10 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1579</v>
+        <v>1639</v>
       </c>
       <c r="D15" s="4" t="n">
         <v>2222</v>
@@ -887,10 +887,10 @@
         <v>14.8</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-28.93789378937894</v>
+        <v>-26.23762376237624</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>33.70025402201524</v>
+        <v>38.78069432684165</v>
       </c>
     </row>
     <row r="16">
@@ -900,10 +900,10 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>30.3</v>
+        <v>34.1</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>353</v>
+        <v>397</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>450</v>
@@ -915,10 +915,10 @@
         <v>12.9</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>-21.55555555555556</v>
+        <v>-11.77777777777778</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>31.71641791044776</v>
+        <v>48.13432835820895</v>
       </c>
     </row>
     <row r="17">
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>20.5</v>
+        <v>20.6</v>
       </c>
       <c r="C17" t="n">
-        <v>1856</v>
+        <v>1863</v>
       </c>
       <c r="D17" t="n">
         <v>1880</v>
@@ -943,10 +943,10 @@
         <v>7.67</v>
       </c>
       <c r="G17" t="n">
-        <v>-1.276595744680851</v>
+        <v>-0.9042553191489361</v>
       </c>
       <c r="H17" t="n">
-        <v>36.17021276595745</v>
+        <v>36.68378576669112</v>
       </c>
     </row>
     <row r="18">
@@ -956,10 +956,10 @@
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>56.8</v>
+        <v>54.9</v>
       </c>
       <c r="C18" s="4" t="n">
-        <v>2484</v>
+        <v>2401</v>
       </c>
       <c r="D18" s="4" t="n">
         <v>3035</v>
@@ -971,10 +971,10 @@
         <v>27.2</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>-18.15485996705107</v>
+        <v>-20.88962108731466</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>14.47004608294931</v>
+        <v>10.64516129032258</v>
       </c>
     </row>
     <row r="19">
@@ -984,10 +984,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>14</v>
+        <v>13.9</v>
       </c>
       <c r="C19" t="n">
-        <v>889</v>
+        <v>879</v>
       </c>
       <c r="D19" t="n">
         <v>922</v>
@@ -999,10 +999,10 @@
         <v>19.7</v>
       </c>
       <c r="G19" t="n">
-        <v>-3.579175704989154</v>
+        <v>-4.663774403470716</v>
       </c>
       <c r="H19" t="n">
-        <v>32.29166666666667</v>
+        <v>30.80357142857143</v>
       </c>
     </row>
     <row r="20">
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>8.119999999999999</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="D20" t="n">
         <v>19.2</v>
@@ -1024,10 +1024,10 @@
         <v>3.6</v>
       </c>
       <c r="G20" t="n">
-        <v>-57.70833333333334</v>
+        <v>-58.17708333333334</v>
       </c>
       <c r="H20" t="n">
-        <v>23.03030303030303</v>
+        <v>21.66666666666666</v>
       </c>
     </row>
     <row r="21">
@@ -1037,10 +1037,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>20.8</v>
+        <v>20.6</v>
       </c>
       <c r="C21" t="n">
-        <v>65.90000000000001</v>
+        <v>65.2</v>
       </c>
       <c r="D21" t="n">
         <v>92.40000000000001</v>
@@ -1052,10 +1052,10 @@
         <v>6.93</v>
       </c>
       <c r="G21" t="n">
-        <v>-28.67965367965368</v>
+        <v>-29.43722943722944</v>
       </c>
       <c r="H21" t="n">
-        <v>11.31756756756757</v>
+        <v>10.13513513513514</v>
       </c>
     </row>
     <row r="22">
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>11.7</v>
+        <v>11.8</v>
       </c>
       <c r="C23" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D23" t="n">
         <v>197</v>
@@ -1108,10 +1108,10 @@
         <v>21.1</v>
       </c>
       <c r="G23" t="n">
-        <v>-27.91878172588833</v>
+        <v>-27.41116751269035</v>
       </c>
       <c r="H23" t="n">
-        <v>21.36752136752137</v>
+        <v>22.22222222222222</v>
       </c>
     </row>
     <row r="24">
@@ -1121,53 +1121,53 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>31.7</v>
+        <v>33.1</v>
       </c>
       <c r="C24" s="3" t="n">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="D24" s="3" t="n">
         <v>229</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>76.8</v>
+        <v>83</v>
       </c>
       <c r="F24" s="3" t="n">
         <v>5.73</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>-31.00436681222708</v>
+        <v>-27.94759825327511</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>105.7291666666667</v>
+        <v>98.79518072289156</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>IRCON</t>
         </is>
       </c>
-      <c r="B25" t="n">
-        <v>23.1</v>
-      </c>
-      <c r="C25" t="n">
-        <v>226</v>
-      </c>
-      <c r="D25" t="n">
+      <c r="B25" s="2" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>236</v>
+      </c>
+      <c r="D25" s="2" t="n">
         <v>352</v>
       </c>
-      <c r="E25" t="n">
+      <c r="E25" s="2" t="n">
         <v>158</v>
       </c>
-      <c r="F25" t="n">
+      <c r="F25" s="2" t="n">
         <v>18.2</v>
       </c>
-      <c r="G25" t="n">
-        <v>-35.79545454545455</v>
-      </c>
-      <c r="H25" t="n">
-        <v>43.03797468354431</v>
+      <c r="G25" s="2" t="n">
+        <v>-32.95454545454545</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>49.36708860759494</v>
       </c>
     </row>
     <row r="26">
@@ -1177,10 +1177,10 @@
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C26" s="4" t="n">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="D26" s="4" t="n">
         <v>395</v>
@@ -1192,10 +1192,10 @@
         <v>1.55</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-14.17721518987342</v>
+        <v>-13.16455696202532</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>48.03493449781659</v>
+        <v>49.78165938864629</v>
       </c>
     </row>
     <row r="27">
@@ -1205,7 +1205,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1389</v>
+        <v>1392</v>
       </c>
       <c r="D27" t="n">
         <v>1635</v>
@@ -1217,10 +1217,10 @@
         <v>0.23</v>
       </c>
       <c r="G27" t="n">
-        <v>-15.04587155963303</v>
+        <v>-14.86238532110092</v>
       </c>
       <c r="H27" t="n">
-        <v>17.61219305673158</v>
+        <v>17.86621507197291</v>
       </c>
     </row>
     <row r="28">
@@ -1230,10 +1230,10 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>18.4</v>
+        <v>18.6</v>
       </c>
       <c r="C28" t="n">
-        <v>1777</v>
+        <v>1795</v>
       </c>
       <c r="D28" t="n">
         <v>1953</v>
@@ -1245,10 +1245,10 @@
         <v>7.86</v>
       </c>
       <c r="G28" t="n">
-        <v>-9.011776753712237</v>
+        <v>-8.090117767537123</v>
       </c>
       <c r="H28" t="n">
-        <v>15.09067357512953</v>
+        <v>16.25647668393782</v>
       </c>
     </row>
     <row r="29">
@@ -1258,10 +1258,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>6.29</v>
+        <v>6.66</v>
       </c>
       <c r="C29" t="n">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="D29" t="n">
         <v>230</v>
@@ -1273,567 +1273,595 @@
         <v>13.8</v>
       </c>
       <c r="G29" t="n">
-        <v>-26.95652173913043</v>
+        <v>-22.60869565217391</v>
       </c>
       <c r="H29" t="n">
-        <v>21.73913043478261</v>
+        <v>28.98550724637681</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>NESTLEIND</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="n">
+        <v>68</v>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>2241</v>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>2778</v>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>2169</v>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>169</v>
+      </c>
+      <c r="G30" s="4" t="n">
+        <v>-19.3304535637149</v>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>3.319502074688797</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>NFL</t>
         </is>
       </c>
-      <c r="B30" t="n">
+      <c r="B31" t="n">
         <v>16.8</v>
       </c>
-      <c r="C30" t="n">
+      <c r="C31" t="n">
         <v>124</v>
       </c>
-      <c r="D30" t="n">
+      <c r="D31" t="n">
         <v>170</v>
       </c>
-      <c r="E30" t="n">
+      <c r="E31" t="n">
         <v>74.8</v>
       </c>
-      <c r="F30" t="n">
+      <c r="F31" t="n">
         <v>6.7</v>
       </c>
-      <c r="G30" t="n">
+      <c r="G31" t="n">
         <v>-27.05882352941176</v>
       </c>
-      <c r="H30" t="n">
+      <c r="H31" t="n">
         <v>65.77540106951872</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>NHPC</t>
         </is>
       </c>
-      <c r="B31" s="2" t="n">
-        <v>28.6</v>
-      </c>
-      <c r="C31" s="2" t="n">
-        <v>84.90000000000001</v>
-      </c>
-      <c r="D31" s="2" t="n">
+      <c r="B32" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>86.09999999999999</v>
+      </c>
+      <c r="D32" s="2" t="n">
         <v>118</v>
       </c>
-      <c r="E31" s="2" t="n">
+      <c r="E32" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="F31" s="2" t="n">
+      <c r="F32" s="2" t="n">
         <v>7.67</v>
       </c>
-      <c r="G31" s="2" t="n">
-        <v>-28.05084745762711</v>
-      </c>
-      <c r="H31" s="2" t="n">
-        <v>46.37931034482759</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>NTPC</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>16.2</v>
-      </c>
-      <c r="C32" t="n">
-        <v>370</v>
-      </c>
-      <c r="D32" t="n">
-        <v>448</v>
-      </c>
-      <c r="E32" t="n">
-        <v>281</v>
-      </c>
-      <c r="F32" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="G32" t="n">
-        <v>-17.41071428571428</v>
-      </c>
-      <c r="H32" t="n">
-        <v>31.67259786476868</v>
+      <c r="G32" s="2" t="n">
+        <v>-27.03389830508475</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>48.44827586206895</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>OIL</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>9.210000000000001</v>
+        <v>16.1</v>
       </c>
       <c r="C33" t="n">
-        <v>475</v>
+        <v>366</v>
       </c>
       <c r="D33" t="n">
-        <v>768</v>
+        <v>448</v>
       </c>
       <c r="E33" t="n">
-        <v>206</v>
+        <v>284</v>
       </c>
       <c r="F33" t="n">
-        <v>17.7</v>
+        <v>10.5</v>
       </c>
       <c r="G33" t="n">
-        <v>-38.15104166666667</v>
+        <v>-18.30357142857143</v>
       </c>
       <c r="H33" t="n">
-        <v>130.5825242718447</v>
+        <v>28.87323943661972</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>OIL</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>9.109999999999999</v>
+      </c>
+      <c r="C34" t="n">
+        <v>470</v>
+      </c>
+      <c r="D34" t="n">
+        <v>768</v>
+      </c>
+      <c r="E34" t="n">
+        <v>206</v>
+      </c>
+      <c r="F34" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-38.80208333333333</v>
+      </c>
+      <c r="H34" t="n">
+        <v>128.1553398058253</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>ONGC</t>
         </is>
       </c>
-      <c r="B34" t="n">
-        <v>7.85</v>
-      </c>
-      <c r="C34" t="n">
-        <v>260</v>
-      </c>
-      <c r="D34" t="n">
+      <c r="B35" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="C35" t="n">
+        <v>257</v>
+      </c>
+      <c r="D35" t="n">
         <v>345</v>
       </c>
-      <c r="E34" t="n">
+      <c r="E35" t="n">
         <v>192</v>
       </c>
-      <c r="F34" t="n">
+      <c r="F35" t="n">
         <v>18.4</v>
       </c>
-      <c r="G34" t="n">
-        <v>-24.63768115942029</v>
-      </c>
-      <c r="H34" t="n">
-        <v>35.41666666666667</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="G35" t="n">
+        <v>-25.50724637681159</v>
+      </c>
+      <c r="H35" t="n">
+        <v>33.85416666666667</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>PIIND</t>
         </is>
       </c>
-      <c r="B35" s="3" t="n">
-        <v>35.4</v>
-      </c>
-      <c r="C35" s="3" t="n">
-        <v>4139</v>
-      </c>
-      <c r="D35" s="3" t="n">
+      <c r="B36" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>4102</v>
+      </c>
+      <c r="D36" s="3" t="n">
         <v>4804</v>
       </c>
-      <c r="E35" s="3" t="n">
+      <c r="E36" s="3" t="n">
         <v>3060</v>
       </c>
-      <c r="F35" s="3" t="n">
+      <c r="F36" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="G35" s="3" t="n">
-        <v>-13.84263114071607</v>
-      </c>
-      <c r="H35" s="3" t="n">
-        <v>35.26143790849673</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>PNB</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>8.75</v>
-      </c>
-      <c r="C36" t="n">
-        <v>110</v>
-      </c>
-      <c r="D36" t="n">
-        <v>143</v>
-      </c>
-      <c r="E36" t="n">
-        <v>84.8</v>
-      </c>
-      <c r="F36" t="n">
-        <v>5.46</v>
-      </c>
-      <c r="G36" t="n">
-        <v>-23.07692307692308</v>
-      </c>
-      <c r="H36" t="n">
-        <v>29.71698113207547</v>
+      <c r="G36" s="3" t="n">
+        <v>-14.61282264779351</v>
+      </c>
+      <c r="H36" s="3" t="n">
+        <v>34.05228758169935</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>8.640000000000001</v>
+      </c>
+      <c r="C37" t="n">
+        <v>109</v>
+      </c>
+      <c r="D37" t="n">
+        <v>143</v>
+      </c>
+      <c r="E37" t="n">
+        <v>84.8</v>
+      </c>
+      <c r="F37" t="n">
+        <v>5.46</v>
+      </c>
+      <c r="G37" t="n">
+        <v>-23.77622377622378</v>
+      </c>
+      <c r="H37" t="n">
+        <v>28.53773584905661</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>PVRINOX</t>
         </is>
       </c>
-      <c r="C37" t="n">
-        <v>1548</v>
-      </c>
-      <c r="D37" t="n">
+      <c r="C38" t="n">
+        <v>1487</v>
+      </c>
+      <c r="D38" t="n">
         <v>1830</v>
       </c>
-      <c r="E37" t="n">
+      <c r="E38" t="n">
         <v>1204</v>
       </c>
-      <c r="F37" t="n">
+      <c r="F38" t="n">
         <v>4.42</v>
       </c>
-      <c r="G37" t="n">
-        <v>-15.40983606557377</v>
-      </c>
-      <c r="H37" t="n">
-        <v>28.57142857142857</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+      <c r="G38" t="n">
+        <v>-18.7431693989071</v>
+      </c>
+      <c r="H38" t="n">
+        <v>23.50498338870432</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>RVNL</t>
         </is>
       </c>
-      <c r="B38" s="4" t="n">
-        <v>71.90000000000001</v>
-      </c>
-      <c r="C38" s="4" t="n">
-        <v>465</v>
-      </c>
-      <c r="D38" s="4" t="n">
+      <c r="B39" s="4" t="n">
+        <v>73.40000000000001</v>
+      </c>
+      <c r="C39" s="4" t="n">
+        <v>474</v>
+      </c>
+      <c r="D39" s="4" t="n">
         <v>647</v>
       </c>
-      <c r="E38" s="4" t="n">
+      <c r="E39" s="4" t="n">
         <v>166</v>
       </c>
-      <c r="F38" s="4" t="n">
+      <c r="F39" s="4" t="n">
         <v>18.4</v>
       </c>
-      <c r="G38" s="4" t="n">
-        <v>-28.12982998454405</v>
-      </c>
-      <c r="H38" s="4" t="n">
-        <v>180.1204819277108</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="G39" s="4" t="n">
+        <v>-26.73879443585781</v>
+      </c>
+      <c r="H39" s="4" t="n">
+        <v>185.5421686746988</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>RELIANCE</t>
         </is>
       </c>
-      <c r="B39" s="2" t="n">
-        <v>26.1</v>
-      </c>
-      <c r="C39" s="2" t="n">
-        <v>1312</v>
-      </c>
-      <c r="D39" s="2" t="n">
+      <c r="B40" s="2" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>1278</v>
+      </c>
+      <c r="D40" s="2" t="n">
         <v>1609</v>
       </c>
-      <c r="E39" s="2" t="n">
+      <c r="E40" s="2" t="n">
         <v>1203</v>
       </c>
-      <c r="F39" s="2" t="n">
+      <c r="F40" s="2" t="n">
         <v>9.609999999999999</v>
       </c>
-      <c r="G39" s="2" t="n">
-        <v>-18.45866998135488</v>
-      </c>
-      <c r="H39" s="2" t="n">
-        <v>9.060681629260182</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>SBICARD</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="n">
-        <v>30.9</v>
-      </c>
-      <c r="C40" s="3" t="n">
-        <v>717</v>
-      </c>
-      <c r="D40" s="3" t="n">
-        <v>817</v>
-      </c>
-      <c r="E40" s="3" t="n">
-        <v>648</v>
-      </c>
-      <c r="F40" s="3" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="G40" s="3" t="n">
-        <v>-12.23990208078335</v>
-      </c>
-      <c r="H40" s="3" t="n">
-        <v>10.64814814814815</v>
+      <c r="G40" s="2" t="n">
+        <v>-20.57178371659416</v>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>6.234413965087282</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
+          <t>SBICARD</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="C41" s="3" t="n">
+        <v>731</v>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>817</v>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>648</v>
+      </c>
+      <c r="F41" s="3" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>-10.52631578947368</v>
+      </c>
+      <c r="H41" s="3" t="n">
+        <v>12.80864197530864</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
           <t>SUPRIYA</t>
         </is>
       </c>
-      <c r="B41" s="3" t="n">
-        <v>39.5</v>
-      </c>
-      <c r="C41" s="3" t="n">
-        <v>774</v>
-      </c>
-      <c r="D41" s="3" t="n">
+      <c r="B42" s="3" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="C42" s="3" t="n">
+        <v>756</v>
+      </c>
+      <c r="D42" s="3" t="n">
         <v>835</v>
       </c>
-      <c r="E41" s="3" t="n">
+      <c r="E42" s="3" t="n">
         <v>269</v>
       </c>
-      <c r="F41" s="3" t="n">
+      <c r="F42" s="3" t="n">
         <v>22.2</v>
       </c>
-      <c r="G41" s="3" t="n">
-        <v>-7.305389221556887</v>
-      </c>
-      <c r="H41" s="3" t="n">
-        <v>187.7323420074349</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>TATAINVEST</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="n">
-        <v>94.7</v>
-      </c>
-      <c r="C42" s="4" t="n">
-        <v>6894</v>
-      </c>
-      <c r="D42" s="4" t="n">
-        <v>9757</v>
-      </c>
-      <c r="E42" s="4" t="n">
-        <v>4013</v>
-      </c>
-      <c r="F42" s="4" t="n">
-        <v>1.67</v>
-      </c>
-      <c r="G42" s="4" t="n">
-        <v>-29.34303576919135</v>
-      </c>
-      <c r="H42" s="4" t="n">
-        <v>71.79167704958883</v>
+      <c r="G42" s="3" t="n">
+        <v>-9.461077844311378</v>
+      </c>
+      <c r="H42" s="3" t="n">
+        <v>181.0408921933085</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
+          <t>TATAINVEST</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="n">
+        <v>95.90000000000001</v>
+      </c>
+      <c r="C43" s="4" t="n">
+        <v>6986</v>
+      </c>
+      <c r="D43" s="4" t="n">
+        <v>9757</v>
+      </c>
+      <c r="E43" s="4" t="n">
+        <v>4013</v>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>-28.40012298862355</v>
+      </c>
+      <c r="H43" s="4" t="n">
+        <v>74.08422626463992</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
           <t>TATAELXSI</t>
         </is>
       </c>
-      <c r="B43" s="4" t="n">
-        <v>451</v>
-      </c>
-      <c r="C43" s="4" t="n">
-        <v>7396</v>
-      </c>
-      <c r="D43" s="4" t="n">
+      <c r="B44" s="4" t="n">
+        <v>449</v>
+      </c>
+      <c r="C44" s="4" t="n">
+        <v>7350</v>
+      </c>
+      <c r="D44" s="4" t="n">
         <v>9200</v>
       </c>
-      <c r="E43" s="4" t="n">
+      <c r="E44" s="4" t="n">
         <v>6285</v>
       </c>
-      <c r="F43" s="4" t="n">
+      <c r="F44" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="G43" s="4" t="n">
-        <v>-19.60869565217391</v>
-      </c>
-      <c r="H43" s="4" t="n">
-        <v>17.67700875099443</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="G44" s="4" t="n">
+        <v>-20.10869565217391</v>
+      </c>
+      <c r="H44" s="4" t="n">
+        <v>16.94510739856802</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
         <is>
           <t>TATAMOTORS</t>
         </is>
       </c>
-      <c r="B44" t="n">
-        <v>8.98</v>
-      </c>
-      <c r="C44" t="n">
-        <v>817</v>
-      </c>
-      <c r="D44" t="n">
+      <c r="B45" t="n">
+        <v>8.789999999999999</v>
+      </c>
+      <c r="C45" t="n">
+        <v>799</v>
+      </c>
+      <c r="D45" t="n">
         <v>1179</v>
       </c>
-      <c r="E44" t="n">
+      <c r="E45" t="n">
         <v>696</v>
       </c>
-      <c r="F44" t="n">
+      <c r="F45" t="n">
         <v>20.1</v>
       </c>
-      <c r="G44" t="n">
-        <v>-30.70398642917727</v>
-      </c>
-      <c r="H44" t="n">
-        <v>17.38505747126437</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>TATAPOWER</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="n">
-        <v>37</v>
-      </c>
-      <c r="C45" s="3" t="n">
-        <v>440</v>
-      </c>
-      <c r="D45" s="3" t="n">
-        <v>495</v>
-      </c>
-      <c r="E45" s="3" t="n">
-        <v>313</v>
-      </c>
-      <c r="F45" s="3" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="G45" s="3" t="n">
-        <v>-11.11111111111111</v>
-      </c>
-      <c r="H45" s="3" t="n">
-        <v>40.57507987220447</v>
+      <c r="G45" t="n">
+        <v>-32.23070398642918</v>
+      </c>
+      <c r="H45" t="n">
+        <v>14.79885057471264</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
+          <t>TATAPOWER</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="C46" s="3" t="n">
+        <v>435</v>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>495</v>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>313</v>
+      </c>
+      <c r="F46" s="3" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="G46" s="3" t="n">
+        <v>-12.12121212121212</v>
+      </c>
+      <c r="H46" s="3" t="n">
+        <v>38.9776357827476</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
           <t>TCS</t>
         </is>
       </c>
-      <c r="B46" s="3" t="n">
-        <v>33.4</v>
-      </c>
-      <c r="C46" s="3" t="n">
-        <v>4446</v>
-      </c>
-      <c r="D46" s="3" t="n">
+      <c r="B47" s="3" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="C47" s="3" t="n">
+        <v>4427</v>
+      </c>
+      <c r="D47" s="3" t="n">
         <v>4592</v>
       </c>
-      <c r="E46" s="3" t="n">
+      <c r="E47" s="3" t="n">
         <v>3563</v>
       </c>
-      <c r="F46" s="3" t="n">
+      <c r="F47" s="3" t="n">
         <v>64.3</v>
       </c>
-      <c r="G46" s="3" t="n">
-        <v>-3.179442508710802</v>
-      </c>
-      <c r="H46" s="3" t="n">
-        <v>24.78248666853775</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
+      <c r="G47" s="3" t="n">
+        <v>-3.593205574912892</v>
+      </c>
+      <c r="H47" s="3" t="n">
+        <v>24.24922817850127</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>TATASTEEL</t>
         </is>
       </c>
-      <c r="B47" s="4" t="n">
-        <v>60.7</v>
-      </c>
-      <c r="C47" s="4" t="n">
-        <v>148</v>
-      </c>
-      <c r="D47" s="4" t="n">
+      <c r="B48" s="4" t="n">
+        <v>61.7</v>
+      </c>
+      <c r="C48" s="4" t="n">
+        <v>151</v>
+      </c>
+      <c r="D48" s="4" t="n">
         <v>185</v>
       </c>
-      <c r="E47" s="4" t="n">
+      <c r="E48" s="4" t="n">
         <v>128</v>
       </c>
-      <c r="F47" s="4" t="n">
+      <c r="F48" s="4" t="n">
         <v>7.02</v>
       </c>
-      <c r="G47" s="4" t="n">
-        <v>-20</v>
-      </c>
-      <c r="H47" s="4" t="n">
-        <v>15.625</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="G48" s="4" t="n">
+        <v>-18.37837837837838</v>
+      </c>
+      <c r="H48" s="4" t="n">
+        <v>17.96875</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>UJJIVANSFB</t>
         </is>
       </c>
-      <c r="B48" t="n">
-        <v>5.83</v>
-      </c>
-      <c r="C48" t="n">
-        <v>35.1</v>
-      </c>
-      <c r="D48" t="n">
-        <v>63</v>
-      </c>
-      <c r="E48" t="n">
+      <c r="B49" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="C49" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="D49" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="E49" t="n">
         <v>32</v>
       </c>
-      <c r="F48" t="n">
+      <c r="F49" t="n">
         <v>11.1</v>
       </c>
-      <c r="G48" t="n">
-        <v>-44.28571428571428</v>
-      </c>
-      <c r="H48" t="n">
-        <v>9.687500000000004</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+      <c r="G49" t="n">
+        <v>-40.93851132686084</v>
+      </c>
+      <c r="H49" t="n">
+        <v>14.0625</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>WIPRO</t>
         </is>
       </c>
-      <c r="B49" s="2" t="n">
-        <v>26.5</v>
-      </c>
-      <c r="C49" s="2" t="n">
-        <v>297</v>
-      </c>
-      <c r="D49" s="2" t="n">
-        <v>301</v>
-      </c>
-      <c r="E49" s="2" t="n">
+      <c r="B50" s="2" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>309</v>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>311</v>
+      </c>
+      <c r="E50" s="2" t="n">
         <v>208</v>
       </c>
-      <c r="F49" s="2" t="n">
+      <c r="F50" s="2" t="n">
         <v>16.9</v>
       </c>
-      <c r="G49" s="2" t="n">
-        <v>-1.32890365448505</v>
-      </c>
-      <c r="H49" s="2" t="n">
-        <v>42.78846153846153</v>
+      <c r="G50" s="2" t="n">
+        <v>-0.6430868167202572</v>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>48.55769230769231</v>
       </c>
     </row>
   </sheetData>

</xml_diff>